<commit_message>
Additional input data edits from custom OBBBA work in eps-us-analysis
</commit_message>
<xml_diff>
--- a/InputData/bldgs/EoDSDwSP/Elasticity of Dist Solar Deployment wrt Subsidy Perc.xlsx
+++ b/InputData/bldgs/EoDSDwSP/Elasticity of Dist Solar Deployment wrt Subsidy Perc.xlsx
@@ -1,22 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Meghan\Dropbox (Energy Innovation)\EPS Versions\eps-1.5.0-us-wipI\InputData\bldgs\EoDSDwSP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us-analysis\InputData\bldgs\EoDSDwSP\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6F7EB30-18B6-4278-8913-DAB4590E9F12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="75" windowWidth="24915" windowHeight="12090"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="Calculations" sheetId="3" r:id="rId2"/>
     <sheet name="EoDSDwSP" sheetId="4" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -89,7 +103,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
@@ -169,9 +183,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -209,9 +223,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -246,7 +260,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -281,7 +295,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -454,16 +468,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -471,37 +485,37 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B4" s="2">
         <v>2015</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -513,17 +527,17 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="35.140625" customWidth="1"/>
-    <col min="3" max="3" width="45.42578125" customWidth="1"/>
-    <col min="4" max="4" width="22.7109375" customWidth="1"/>
+    <col min="2" max="2" width="35.1796875" customWidth="1"/>
+    <col min="3" max="3" width="45.453125" customWidth="1"/>
+    <col min="4" max="4" width="22.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -537,7 +551,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -552,7 +566,7 @@
         <v>0.43949044585987279</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -567,12 +581,12 @@
         <v>0.37984496124031009</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>0.3</v>
       </c>
@@ -580,12 +594,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -594,7 +608,7 @@
         <v>1.4649681528662426</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -610,46 +624,43 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.140625" customWidth="1"/>
+    <col min="1" max="1" width="22.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>15</v>
       </c>
       <c r="B2" s="6">
-        <f>Calculations!B9</f>
-        <v>1.4649681528662426</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>16</v>
       </c>
       <c r="B3" s="6">
-        <f>B2</f>
-        <v>1.4649681528662426</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="6">
-        <f>Calculations!B10</f>
-        <v>1.2661498708010337</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Swaps to using endogenous solar deployment for 25D in frozen policy & climate ambition scenarios; uses CiDESCTY to represent Solar for All
</commit_message>
<xml_diff>
--- a/InputData/bldgs/EoDSDwSP/Elasticity of Dist Solar Deployment wrt Subsidy Perc.xlsx
+++ b/InputData/bldgs/EoDSDwSP/Elasticity of Dist Solar Deployment wrt Subsidy Perc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us-analysis\InputData\bldgs\EoDSDwSP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\bldgs\EoDSDwSP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6F7EB30-18B6-4278-8913-DAB4590E9F12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B7E60EC-3329-461B-BAA2-DC75E0655131}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-26430" yWindow="1485" windowWidth="26400" windowHeight="14490" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -470,14 +470,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -485,37 +485,37 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" s="2">
         <v>2015</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -529,15 +529,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="35.1796875" customWidth="1"/>
-    <col min="3" max="3" width="45.453125" customWidth="1"/>
-    <col min="4" max="4" width="22.7265625" customWidth="1"/>
+    <col min="2" max="2" width="35.140625" customWidth="1"/>
+    <col min="3" max="3" width="45.42578125" customWidth="1"/>
+    <col min="4" max="4" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -551,7 +551,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -566,7 +566,7 @@
         <v>0.43949044585987279</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -581,12 +581,12 @@
         <v>0.37984496124031009</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>0.3</v>
       </c>
@@ -594,12 +594,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -608,7 +608,7 @@
         <v>1.4649681528662426</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -629,38 +629,41 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.1796875" customWidth="1"/>
+    <col min="1" max="1" width="22.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>15</v>
       </c>
       <c r="B2" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+        <f>Calculations!B9</f>
+        <v>1.4649681528662426</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>16</v>
       </c>
       <c r="B3" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+        <f>Calculations!B9</f>
+        <v>1.4649681528662426</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="6">
-        <v>0</v>
+        <f>Calculations!B10</f>
+        <v>1.2661498708010337</v>
       </c>
     </row>
   </sheetData>

</xml_diff>